<commit_message>
feat: Add FastAPI backend for PDF purchase order data extraction and Excel tracker management.
</commit_message>
<xml_diff>
--- a/Blinkit PO Tracker.xlsx
+++ b/Blinkit PO Tracker.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG2"/>
+  <dimension ref="A1:AG4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.140625" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -697,6 +697,92 @@
         <v>2898</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Zomato Hyperpure Private Limited</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Jaipur J3 Feeder warehouse</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>487</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MANOJ SOAP AGENCY-JAIPUR</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>6478810007248</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>46070</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Shareat Whole Wheat Foochka Pani Puri(Packet) (200 g)</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>120</v>
+      </c>
+      <c r="O3" t="n">
+        <v>24.15</v>
+      </c>
+      <c r="P3" t="n">
+        <v>2898</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Zomato Hyperpure Private Limited</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jaipur J3 Feeder warehouse</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>487</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>MANOJ SOAP AGENCY-JAIPUR</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>6478810007248</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>46070</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Shareat Whole Wheat Foochka Pani Puri(Packet) (200 g)</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>120</v>
+      </c>
+      <c r="O4" t="n">
+        <v>24.15</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2898</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1:XFD1">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>

<commit_message>
feat: Implement a FastAPI backend with PDF PO data extraction and Excel tracker management capabilities.
</commit_message>
<xml_diff>
--- a/Blinkit PO Tracker.xlsx
+++ b/Blinkit PO Tracker.xlsx
@@ -15,9 +15,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD-MMM-YYYY"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -448,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.140625" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -654,135 +653,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Zomato Hyperpure Private Limited</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Jaipur J3 Feeder warehouse</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>487</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>MANOJ SOAP AGENCY-JAIPUR</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>6478810007248</v>
-      </c>
-      <c r="H2" s="9" t="n">
-        <v>46070</v>
-      </c>
-      <c r="I2" s="9" t="n">
-        <v>46080</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Shareat Whole Wheat Foochka Pani Puri(Packet) (200 g)</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>120</v>
-      </c>
-      <c r="O2" t="n">
-        <v>24.15</v>
-      </c>
-      <c r="P2" t="n">
-        <v>2898</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Zomato Hyperpure Private Limited</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Jaipur J3 Feeder warehouse</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>487</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MANOJ SOAP AGENCY-JAIPUR</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>6478810007248</v>
-      </c>
-      <c r="H3" s="9" t="n">
-        <v>46070</v>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>46080</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Shareat Whole Wheat Foochka Pani Puri(Packet) (200 g)</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>120</v>
-      </c>
-      <c r="O3" t="n">
-        <v>24.15</v>
-      </c>
-      <c r="P3" t="n">
-        <v>2898</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Zomato Hyperpure Private Limited</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Jaipur J3 Feeder warehouse</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>487</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>MANOJ SOAP AGENCY-JAIPUR</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>6478810007248</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>46070</v>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>46080</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Shareat Whole Wheat Foochka Pani Puri(Packet) (200 g)</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>120</v>
-      </c>
-      <c r="O4" t="n">
-        <v>24.15</v>
-      </c>
-      <c r="P4" t="n">
-        <v>2898</v>
-      </c>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="A1:XFD1">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>